<commit_message>
add upgrade sprites to tower_upgrades.pdf
</commit_message>
<xml_diff>
--- a/assets/tower_upgrades.xlsx
+++ b/assets/tower_upgrades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daten\Projekte\pico\pico-bubble-towers\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760F1EC1-9294-40CD-B72F-CE95BCE43997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377077C8-2F05-41CA-A015-93748907DB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{4E8ABA74-1C8E-408B-B6B2-4FB773843FD4}"/>
   </bookViews>
@@ -204,22 +204,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="15">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -234,17 +223,46 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
-      </right>
-      <top style="thin">
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
@@ -254,7 +272,7 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -262,7 +280,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
@@ -274,7 +292,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -283,11 +303,53 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -296,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -308,91 +370,106 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -426,13 +503,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>4483</xdr:colOff>
+      <xdr:colOff>14008</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>195471</xdr:rowOff>
     </xdr:to>
@@ -462,8 +539,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="605118" y="212912"/>
-          <a:ext cx="609600" cy="621295"/>
+          <a:off x="619125" y="628650"/>
+          <a:ext cx="614083" cy="614571"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -673,13 +750,13 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>16329</xdr:rowOff>
+      <xdr:rowOff>1675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>1</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>209549</xdr:rowOff>
+      <xdr:rowOff>194895</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -707,8 +784,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5446059" y="1932535"/>
-          <a:ext cx="605118" cy="622406"/>
+          <a:off x="5180135" y="4251290"/>
+          <a:ext cx="608135" cy="618182"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1197,8 +1274,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2895600" y="9764486"/>
-          <a:ext cx="609372" cy="631371"/>
+          <a:off x="2896914" y="9669517"/>
+          <a:ext cx="609372" cy="627242"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1883,8 +1960,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4038600" y="9764486"/>
-          <a:ext cx="609372" cy="631371"/>
+          <a:off x="4039914" y="9669517"/>
+          <a:ext cx="609372" cy="627242"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1932,8 +2009,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5181600" y="9764486"/>
-          <a:ext cx="609372" cy="631371"/>
+          <a:off x="5182914" y="9669517"/>
+          <a:ext cx="609372" cy="627242"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2281,6 +2358,2189 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3923</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>194221</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>231055</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>4333</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Grafik 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08B140EF-90E3-8325-80D4-92B4C6CA88EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="37908" r="81209" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1755058" y="3806394"/>
+          <a:ext cx="227132" cy="235074"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>7843</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>180165</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>246639</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>202759</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Grafik 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA77C040-5BBD-4575-957B-8D3A9B00A946}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18586" t="37908" r="74889" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1758978" y="8466915"/>
+          <a:ext cx="238796" cy="235075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>198</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>186042</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>222799</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>202121</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Grafik 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{599F27A5-5A83-4009-B991-3A2790C14BAA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2897112" y="10065766"/>
+          <a:ext cx="222601" cy="226286"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>531356</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>189510</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>226846</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>202391</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Grafik 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B73928B7-35A7-41BB-96D6-292B85405C55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2890625" y="8476260"/>
+          <a:ext cx="230356" cy="225362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>5964</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>17234</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>204120</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>6501</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Grafik 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43B62B6C-6807-467E-A26E-55050D6C6EFF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2900099" y="3841888"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>532038</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>15768</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>195328</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>5035</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="37" name="Grafik 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECC4BF2C-A374-4616-8320-B705F8F8A1A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4034307" y="3840422"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3034</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>16186</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>201190</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>5453</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="Grafik 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1B831DA-3C97-45D7-82BE-EDDAC79E1CBD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5184634" y="3837072"/>
+          <a:ext cx="198156" cy="201538"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1134</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>179473</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>231490</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>192354</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="Grafik 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D834E3C-4E78-41AB-8967-DFDBB5152D7C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2896734" y="4637173"/>
+          <a:ext cx="230356" cy="225152"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1134</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>181776</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>230024</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>194657</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="Grafik 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9714696C-8B57-4BAC-8C41-2CD6C59C5FCA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4039734" y="4639476"/>
+          <a:ext cx="228890" cy="225152"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>533068</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>185754</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228558</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>198635</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Grafik 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4FB768D-B067-47E9-A56E-210F9C1C993E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5178337" y="4647850"/>
+          <a:ext cx="230356" cy="225362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>533504</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>200407</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>196794</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>189674</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Grafik 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5E9B213-0BC5-4840-8294-359940A42CEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1749773" y="1050330"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>532039</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>195174</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>195329</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>184441</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="43" name="Grafik 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2F8147F-15BC-4DD0-9D59-B7655399E70B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2894239" y="1044260"/>
+          <a:ext cx="196690" cy="201538"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3035</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>204804</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>201191</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>194071</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="44" name="Grafik 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDF6AFFB-1879-4A33-9921-7ED425561409}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4040170" y="1054727"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1570</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>201455</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>199726</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>190722</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="45" name="Grafik 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3996E361-1729-49B6-A415-99EA548ECCFC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5183170" y="1050541"/>
+          <a:ext cx="198156" cy="201538"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>8461</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>184287</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>233842</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>200366</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="46" name="Grafik 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CDFFFAA-FBC9-4239-9CBC-B94D3D733AD5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2902596" y="1884133"/>
+          <a:ext cx="225381" cy="228560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>6995</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>182821</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>232376</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>198900</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="49" name="Grafik 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A4C43E3-97B7-45E0-B813-DAEB5DF807FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4044130" y="1882667"/>
+          <a:ext cx="225381" cy="228560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>533069</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>181355</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>223584</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>197434</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Grafik 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EA87631-37AC-4EA4-A55B-218296EC8DA7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5178338" y="1881201"/>
+          <a:ext cx="225381" cy="228560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3018</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>184916</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>233374</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>197797</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Grafik 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4129118A-26E5-49E4-9579-1DF4E9C13556}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2898618" y="2732173"/>
+          <a:ext cx="230356" cy="225153"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1134</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>185334</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>230024</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>198215</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="Grafik 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC5A669F-21FA-4C0A-8A52-0FDBDA5C764B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4039734" y="2732591"/>
+          <a:ext cx="228890" cy="225153"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>533068</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>185752</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228558</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>198633</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Grafik 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7531720E-5FA2-4E2F-84DB-1AA14DB48B0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5178337" y="2735521"/>
+          <a:ext cx="230356" cy="225362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>532698</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>166497</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>230334</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>192288</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Grafik 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF581104-5DB3-4A60-A831-FBFFFFB49C89}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="24906" t="37908" r="68716" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1751898" y="5685554"/>
+          <a:ext cx="231036" cy="238063"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>533503</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>200407</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>196793</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>189674</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="55" name="Grafik 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34C72C39-A540-446A-9E8D-2E47F1203184}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2892772" y="5724907"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>532037</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>206269</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>195327</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>195536</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="60" name="Grafik 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E79214F-5214-480C-9821-CE87002BC112}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4034306" y="5730769"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3032</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>207118</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>201188</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>196385</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="61" name="Grafik 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{791D4D5A-55F2-422A-B106-911ADE70252F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5186637" y="5681486"/>
+          <a:ext cx="198156" cy="199820"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>531357</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>190149</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>224554</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>203029</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="67" name="Grafik 66">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57B9E449-8A19-4371-94AC-10A75AF57C73}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="24994" t="44217" r="68775" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2890626" y="7414495"/>
+          <a:ext cx="228063" cy="225361"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2353</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>186800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>230416</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>199680</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="68" name="Grafik 67">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{469170D2-76AA-4875-99EE-4D20380BB633}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="24994" t="44217" r="68775" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4040953" y="7404029"/>
+          <a:ext cx="228063" cy="225151"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>887</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>187977</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228950</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>200857</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="70" name="Grafik 69">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B79B04B-5C70-4ED8-A333-FD65051973D3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="24994" t="44217" r="68775" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5183801" y="7335011"/>
+          <a:ext cx="228063" cy="223087"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>534350</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>180641</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>223256</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>203235</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="71" name="Grafik 70">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B30A445-F6E0-4383-90A9-FA931D569677}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31372" t="37908" r="62514" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2893619" y="6555064"/>
+          <a:ext cx="223772" cy="235075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>532884</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>179176</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>221790</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>201770</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="72" name="Grafik 71">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC96D521-9BF0-46C5-BA29-3FDA14DD22EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31372" t="37908" r="62514" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4035153" y="6553599"/>
+          <a:ext cx="223772" cy="235075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>531418</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>179595</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>220324</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>202189</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="73" name="Grafik 72">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40B4A988-1EB0-4274-80B6-898E06A74E33}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31372" t="37908" r="62514" b="55797"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5179618" y="6547738"/>
+          <a:ext cx="222306" cy="234865"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2351</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>188045</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>232707</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>200926</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="74" name="Grafik 73">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83C78130-F589-4CDB-924C-6ECF3062FDB3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4039486" y="8474795"/>
+          <a:ext cx="230356" cy="225362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>885</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>193907</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>231241</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>206788</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="75" name="Grafik 74">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA6B39F6-70DA-4408-AD1A-5E6E8B7FC16E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="31166" t="44217" r="62514" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5181020" y="8480657"/>
+          <a:ext cx="230356" cy="225362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3279</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>184577</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>228660</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>200656</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="77" name="Grafik 76">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDB1CE14-1628-41BD-809D-D52A57FBF6C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4040414" y="10171173"/>
+          <a:ext cx="225381" cy="228560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3697</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>190439</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>229078</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>206518</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="78" name="Grafik 77">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42BA3CDB-E441-4278-AD37-80E262C76B98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="18674" t="44217" r="75168" b="49752"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5185297" y="10167196"/>
+          <a:ext cx="225381" cy="228351"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1714</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>200695</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>199870</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>189962</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="79" name="Grafik 78">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB03677F-33DB-4CE5-B267-190E27605E69}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2895849" y="9337368"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>249</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>199230</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>198405</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>188497</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="80" name="Grafik 79">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D0B3417-215F-4DE5-99EC-2EA5D6ADE421}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4037384" y="9335903"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>533650</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>197765</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>196940</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>187032</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="81" name="Grafik 80">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13E13230-7954-48D3-A6C6-A57DB4E912A6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="12560" t="44217" r="82001" b="50393"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5178919" y="9334438"/>
+          <a:ext cx="198156" cy="201748"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2614,67 +4874,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="28">
+      <c r="B1" s="16">
         <v>0</v>
       </c>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28">
+      <c r="C1" s="16"/>
+      <c r="D1" s="16">
         <v>1</v>
       </c>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28">
+      <c r="E1" s="16"/>
+      <c r="F1" s="16">
         <v>2</v>
       </c>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28">
+      <c r="G1" s="16"/>
+      <c r="H1" s="16">
         <v>3</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28">
+      <c r="I1" s="16"/>
+      <c r="J1" s="16">
         <v>4</v>
       </c>
-      <c r="K1" s="28"/>
+      <c r="K1" s="16"/>
     </row>
-    <row r="2" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+    <row r="2" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
     </row>
     <row r="3" spans="1:23" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="37">
         <v>10</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24">
+      <c r="C3" s="38"/>
+      <c r="D3" s="38">
         <v>18</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24">
+      <c r="E3" s="38"/>
+      <c r="F3" s="38">
         <v>32</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24">
+      <c r="G3" s="38"/>
+      <c r="H3" s="38">
         <v>90</v>
       </c>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24">
+      <c r="I3" s="38"/>
+      <c r="J3" s="38">
         <v>225</v>
       </c>
-      <c r="K3" s="25"/>
+      <c r="K3" s="39"/>
       <c r="M3" s="3"/>
       <c r="O3" s="3"/>
       <c r="Q3" s="3"/>
@@ -2686,24 +4946,24 @@
       <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9">
+      <c r="B4" s="21"/>
+      <c r="C4" s="6">
         <v>10</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="9">
+      <c r="D4" s="7"/>
+      <c r="E4" s="6">
         <v>15</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9">
+      <c r="F4" s="7"/>
+      <c r="G4" s="6">
         <v>25</v>
       </c>
-      <c r="H4" s="10"/>
-      <c r="I4" s="9">
+      <c r="H4" s="7"/>
+      <c r="I4" s="6">
         <v>50</v>
       </c>
-      <c r="J4" s="10"/>
-      <c r="K4" s="11">
+      <c r="J4" s="7"/>
+      <c r="K4" s="22">
         <v>70</v>
       </c>
     </row>
@@ -2711,24 +4971,24 @@
       <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9">
+      <c r="B5" s="21"/>
+      <c r="C5" s="6">
         <v>16</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9">
+      <c r="D5" s="7"/>
+      <c r="E5" s="6">
         <v>18.600000000000001</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9">
+      <c r="F5" s="7"/>
+      <c r="G5" s="6">
         <v>21.3</v>
       </c>
-      <c r="H5" s="10"/>
-      <c r="I5" s="9">
+      <c r="H5" s="7"/>
+      <c r="I5" s="6">
         <v>26.6</v>
       </c>
-      <c r="J5" s="10"/>
-      <c r="K5" s="11">
+      <c r="J5" s="7"/>
+      <c r="K5" s="22">
         <v>60</v>
       </c>
     </row>
@@ -2736,812 +4996,812 @@
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="9">
+      <c r="B6" s="21"/>
+      <c r="C6" s="6">
         <v>10</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="9">
+      <c r="D6" s="7"/>
+      <c r="E6" s="6">
         <v>10</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9">
+      <c r="F6" s="7"/>
+      <c r="G6" s="6">
         <v>10</v>
       </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="9">
+      <c r="H6" s="7"/>
+      <c r="I6" s="6">
         <v>10</v>
       </c>
-      <c r="J6" s="10"/>
-      <c r="K6" s="11">
+      <c r="J6" s="7"/>
+      <c r="K6" s="22">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9">
+      <c r="B7" s="34"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6">
         <v>40</v>
       </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9">
+      <c r="G7" s="6"/>
+      <c r="H7" s="6">
         <v>100</v>
       </c>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9">
+      <c r="I7" s="6"/>
+      <c r="J7" s="6">
         <v>190</v>
       </c>
-      <c r="K7" s="11"/>
+      <c r="K7" s="22"/>
     </row>
     <row r="8" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10" t="s">
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9">
+      <c r="F8" s="7"/>
+      <c r="G8" s="6">
         <v>20</v>
       </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="9">
+      <c r="H8" s="7"/>
+      <c r="I8" s="6">
         <v>35</v>
       </c>
-      <c r="J8" s="9"/>
-      <c r="K8" s="11">
+      <c r="J8" s="6"/>
+      <c r="K8" s="22">
         <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10" t="s">
+      <c r="C9" s="6"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9">
+      <c r="F9" s="7"/>
+      <c r="G9" s="6">
         <v>18.600000000000001</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="9">
+      <c r="H9" s="7"/>
+      <c r="I9" s="6">
         <v>21.3</v>
       </c>
-      <c r="J9" s="9"/>
-      <c r="K9" s="11">
+      <c r="J9" s="6"/>
+      <c r="K9" s="22">
         <v>26.6</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15" t="s">
+      <c r="B10" s="23"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="14">
+      <c r="F10" s="9"/>
+      <c r="G10" s="8">
         <v>6.6</v>
       </c>
-      <c r="H10" s="15"/>
-      <c r="I10" s="14">
+      <c r="H10" s="9"/>
+      <c r="I10" s="8">
         <v>5.3</v>
       </c>
-      <c r="J10" s="14"/>
-      <c r="K10" s="16">
+      <c r="J10" s="8"/>
+      <c r="K10" s="24">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5">
         <v>50</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6">
+      <c r="G11" s="5"/>
+      <c r="H11" s="5">
         <v>115</v>
       </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6">
+      <c r="I11" s="5"/>
+      <c r="J11" s="5">
         <v>150</v>
       </c>
-      <c r="K11" s="7"/>
+      <c r="K11" s="25"/>
     </row>
     <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="9">
+      <c r="F12" s="7"/>
+      <c r="G12" s="6">
         <v>35</v>
       </c>
-      <c r="H12" s="10"/>
-      <c r="I12" s="9">
+      <c r="H12" s="7"/>
+      <c r="I12" s="6">
         <v>75</v>
       </c>
-      <c r="J12" s="10"/>
-      <c r="K12" s="11">
+      <c r="J12" s="7"/>
+      <c r="K12" s="22">
         <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10" t="s">
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="9">
+      <c r="F13" s="7"/>
+      <c r="G13" s="6">
         <v>21.3</v>
       </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="9">
+      <c r="H13" s="7"/>
+      <c r="I13" s="6">
         <v>24</v>
       </c>
-      <c r="J13" s="10"/>
-      <c r="K13" s="11">
+      <c r="J13" s="7"/>
+      <c r="K13" s="22">
         <v>29.3</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15" t="s">
+      <c r="C14" s="30"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="F14" s="15"/>
-      <c r="G14" s="14">
+      <c r="F14" s="31"/>
+      <c r="G14" s="30">
         <v>13.3</v>
       </c>
-      <c r="H14" s="15"/>
-      <c r="I14" s="14">
+      <c r="H14" s="31"/>
+      <c r="I14" s="30">
         <v>13.3</v>
       </c>
-      <c r="J14" s="15"/>
-      <c r="K14" s="16">
+      <c r="J14" s="31"/>
+      <c r="K14" s="35">
         <v>13.3</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
     </row>
     <row r="16" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6">
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19">
         <v>20</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6">
+      <c r="E16" s="19"/>
+      <c r="F16" s="19">
         <v>40</v>
       </c>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6">
+      <c r="G16" s="19"/>
+      <c r="H16" s="19">
         <v>100</v>
       </c>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6">
+      <c r="I16" s="19"/>
+      <c r="J16" s="19">
         <v>250</v>
       </c>
-      <c r="K16" s="7"/>
+      <c r="K16" s="20"/>
     </row>
     <row r="17" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="8"/>
-      <c r="C17" s="10" t="s">
+      <c r="B17" s="21"/>
+      <c r="C17" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="9">
+      <c r="D17" s="7"/>
+      <c r="E17" s="6">
         <v>20</v>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="9">
+      <c r="F17" s="7"/>
+      <c r="G17" s="6">
         <v>30</v>
       </c>
-      <c r="H17" s="10"/>
-      <c r="I17" s="9">
+      <c r="H17" s="7"/>
+      <c r="I17" s="6">
         <v>50</v>
       </c>
-      <c r="J17" s="10"/>
-      <c r="K17" s="11">
+      <c r="J17" s="7"/>
+      <c r="K17" s="22">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="8"/>
-      <c r="C18" s="10" t="s">
+      <c r="B18" s="21"/>
+      <c r="C18" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D18" s="10"/>
-      <c r="E18" s="9">
+      <c r="D18" s="7"/>
+      <c r="E18" s="6">
         <v>24</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="9">
+      <c r="F18" s="7"/>
+      <c r="G18" s="6">
         <v>26.6</v>
       </c>
-      <c r="H18" s="10"/>
-      <c r="I18" s="9">
+      <c r="H18" s="7"/>
+      <c r="I18" s="6">
         <v>33.299999999999997</v>
       </c>
-      <c r="J18" s="10"/>
-      <c r="K18" s="11">
+      <c r="J18" s="7"/>
+      <c r="K18" s="22">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="10" t="s">
+      <c r="B19" s="21"/>
+      <c r="C19" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="9">
+      <c r="D19" s="7"/>
+      <c r="E19" s="6">
         <v>10</v>
       </c>
-      <c r="F19" s="10"/>
-      <c r="G19" s="9">
+      <c r="F19" s="7"/>
+      <c r="G19" s="6">
         <v>10</v>
       </c>
-      <c r="H19" s="10"/>
-      <c r="I19" s="9">
+      <c r="H19" s="7"/>
+      <c r="I19" s="6">
         <v>10</v>
       </c>
-      <c r="J19" s="10"/>
-      <c r="K19" s="11">
+      <c r="J19" s="7"/>
+      <c r="K19" s="22">
         <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9">
+      <c r="B20" s="34"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6">
         <v>50</v>
       </c>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9">
+      <c r="G20" s="6"/>
+      <c r="H20" s="6">
         <v>130</v>
       </c>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9">
+      <c r="I20" s="6"/>
+      <c r="J20" s="6">
         <v>325</v>
       </c>
-      <c r="K20" s="11"/>
+      <c r="K20" s="22"/>
     </row>
     <row r="21" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10" t="s">
+      <c r="C21" s="6"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="9">
+      <c r="F21" s="7"/>
+      <c r="G21" s="6">
         <v>40</v>
       </c>
-      <c r="H21" s="10"/>
-      <c r="I21" s="9">
+      <c r="H21" s="7"/>
+      <c r="I21" s="6">
         <v>60</v>
       </c>
-      <c r="J21" s="10"/>
-      <c r="K21" s="11">
+      <c r="J21" s="7"/>
+      <c r="K21" s="22">
         <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10" t="s">
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="9">
+      <c r="F22" s="7"/>
+      <c r="G22" s="6">
         <v>18.600000000000001</v>
       </c>
-      <c r="H22" s="10"/>
-      <c r="I22" s="9">
+      <c r="H22" s="7"/>
+      <c r="I22" s="6">
         <v>24</v>
       </c>
-      <c r="J22" s="10"/>
-      <c r="K22" s="11">
+      <c r="J22" s="7"/>
+      <c r="K22" s="22">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15" t="s">
+      <c r="C23" s="30"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="F23" s="15"/>
-      <c r="G23" s="14">
+      <c r="F23" s="31"/>
+      <c r="G23" s="30">
         <v>13.3</v>
       </c>
-      <c r="H23" s="15"/>
-      <c r="I23" s="14">
+      <c r="H23" s="31"/>
+      <c r="I23" s="30">
         <v>13.3</v>
       </c>
-      <c r="J23" s="15"/>
-      <c r="K23" s="16">
+      <c r="J23" s="31"/>
+      <c r="K23" s="35">
         <v>13.3</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6">
+      <c r="C25" s="19"/>
+      <c r="D25" s="19">
         <v>35</v>
       </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6">
+      <c r="E25" s="19"/>
+      <c r="F25" s="19">
         <v>50</v>
       </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6">
+      <c r="G25" s="19"/>
+      <c r="H25" s="19">
         <v>115</v>
       </c>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6">
+      <c r="I25" s="19"/>
+      <c r="J25" s="19">
         <v>350</v>
       </c>
-      <c r="K25" s="7"/>
+      <c r="K25" s="20"/>
     </row>
     <row r="26" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="8"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="9">
+      <c r="B26" s="21"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="6">
         <v>15</v>
       </c>
-      <c r="F26" s="10"/>
-      <c r="G26" s="9">
+      <c r="F26" s="7"/>
+      <c r="G26" s="6">
         <v>20</v>
       </c>
-      <c r="H26" s="10"/>
-      <c r="I26" s="9">
+      <c r="H26" s="7"/>
+      <c r="I26" s="6">
         <v>50</v>
       </c>
-      <c r="J26" s="10"/>
-      <c r="K26" s="11">
+      <c r="J26" s="7"/>
+      <c r="K26" s="22">
         <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="9">
+      <c r="B27" s="21"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="6">
         <v>13.3</v>
       </c>
-      <c r="F27" s="10"/>
-      <c r="G27" s="9">
+      <c r="F27" s="7"/>
+      <c r="G27" s="6">
         <v>16</v>
       </c>
-      <c r="H27" s="10"/>
-      <c r="I27" s="9">
+      <c r="H27" s="7"/>
+      <c r="I27" s="6">
         <v>18.600000000000001</v>
       </c>
-      <c r="J27" s="10"/>
-      <c r="K27" s="11">
+      <c r="J27" s="7"/>
+      <c r="K27" s="22">
         <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="14">
+      <c r="B28" s="23"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="8">
         <v>10</v>
       </c>
-      <c r="F28" s="15"/>
-      <c r="G28" s="14">
+      <c r="F28" s="9"/>
+      <c r="G28" s="8">
         <v>10</v>
       </c>
-      <c r="H28" s="15"/>
-      <c r="I28" s="14">
+      <c r="H28" s="9"/>
+      <c r="I28" s="8">
         <v>10</v>
       </c>
-      <c r="J28" s="15"/>
-      <c r="K28" s="16">
+      <c r="J28" s="9"/>
+      <c r="K28" s="24">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6">
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5">
         <v>80</v>
       </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6">
+      <c r="G29" s="5"/>
+      <c r="H29" s="5">
         <v>130</v>
       </c>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6">
+      <c r="I29" s="5"/>
+      <c r="J29" s="5">
         <v>220</v>
       </c>
-      <c r="K29" s="7"/>
+      <c r="K29" s="25"/>
     </row>
     <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="9"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="21" t="s">
+      <c r="C30" s="6"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="F30" s="10"/>
-      <c r="G30" s="21" t="s">
+      <c r="F30" s="7"/>
+      <c r="G30" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H30" s="10"/>
-      <c r="I30" s="21" t="s">
+      <c r="H30" s="7"/>
+      <c r="I30" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J30" s="10"/>
-      <c r="K30" s="22" t="s">
+      <c r="J30" s="7"/>
+      <c r="K30" s="26" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="21" t="s">
+      <c r="C31" s="6"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="F31" s="10"/>
-      <c r="G31" s="21">
+      <c r="F31" s="7"/>
+      <c r="G31" s="11">
         <v>14</v>
       </c>
-      <c r="H31" s="10"/>
-      <c r="I31" s="21">
+      <c r="H31" s="7"/>
+      <c r="I31" s="11">
         <v>16</v>
       </c>
-      <c r="J31" s="10"/>
-      <c r="K31" s="22">
+      <c r="J31" s="7"/>
+      <c r="K31" s="26">
         <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="13"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="15"/>
-      <c r="K32" s="16"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="24"/>
     </row>
     <row r="33" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6">
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5">
         <v>35</v>
       </c>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6">
+      <c r="G33" s="5"/>
+      <c r="H33" s="5">
         <v>90</v>
       </c>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6">
+      <c r="I33" s="5"/>
+      <c r="J33" s="5">
         <v>180</v>
       </c>
-      <c r="K33" s="7"/>
+      <c r="K33" s="25"/>
     </row>
     <row r="34" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="9"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="11"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="22"/>
     </row>
     <row r="35" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C35" s="9"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="17" t="s">
+      <c r="C35" s="6"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F35" s="10"/>
-      <c r="G35" s="17">
+      <c r="F35" s="7"/>
+      <c r="G35" s="10">
         <v>14</v>
       </c>
-      <c r="H35" s="10"/>
-      <c r="I35" s="17">
+      <c r="H35" s="7"/>
+      <c r="I35" s="10">
         <v>18.600000000000001</v>
       </c>
-      <c r="J35" s="10"/>
-      <c r="K35" s="18">
+      <c r="J35" s="7"/>
+      <c r="K35" s="28">
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="13"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="19" t="s">
+    <row r="36" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="29"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="F36" s="15"/>
-      <c r="G36" s="19" t="s">
+      <c r="F36" s="31"/>
+      <c r="G36" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="H36" s="15"/>
-      <c r="I36" s="19" t="s">
+      <c r="H36" s="31"/>
+      <c r="I36" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="J36" s="15"/>
-      <c r="K36" s="20" t="s">
+      <c r="J36" s="31"/>
+      <c r="K36" s="33" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="38" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="5"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6">
+      <c r="B38" s="18"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19">
         <v>40</v>
       </c>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6">
+      <c r="E38" s="19"/>
+      <c r="F38" s="19">
         <v>50</v>
       </c>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6">
+      <c r="G38" s="19"/>
+      <c r="H38" s="19">
         <v>90</v>
       </c>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6">
+      <c r="I38" s="19"/>
+      <c r="J38" s="19">
         <v>190</v>
       </c>
-      <c r="K38" s="7"/>
+      <c r="K38" s="20"/>
     </row>
     <row r="39" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="8"/>
-      <c r="C39" s="35" t="s">
+      <c r="B39" s="21"/>
+      <c r="C39" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="D39" s="10"/>
-      <c r="E39" s="36" t="s">
+      <c r="D39" s="7"/>
+      <c r="E39" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F39" s="10"/>
-      <c r="G39" s="36" t="s">
+      <c r="F39" s="7"/>
+      <c r="G39" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="10"/>
-      <c r="I39" s="36" t="s">
+      <c r="H39" s="7"/>
+      <c r="I39" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J39" s="10"/>
-      <c r="K39" s="37" t="s">
+      <c r="J39" s="7"/>
+      <c r="K39" s="41" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="40" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="8"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="10"/>
-      <c r="K40" s="11"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="22"/>
     </row>
     <row r="41" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="8"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="10"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="11"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="22"/>
     </row>
     <row r="42" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="12"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9">
+      <c r="B42" s="34"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6">
         <v>40</v>
       </c>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9">
+      <c r="G42" s="6"/>
+      <c r="H42" s="6">
         <v>75</v>
       </c>
-      <c r="I42" s="9"/>
-      <c r="J42" s="9">
+      <c r="I42" s="6"/>
+      <c r="J42" s="6">
         <v>175</v>
       </c>
-      <c r="K42" s="11"/>
+      <c r="K42" s="22"/>
     </row>
     <row r="43" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="11"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="7"/>
+      <c r="K43" s="22"/>
     </row>
     <row r="44" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C44" s="9"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="31" t="s">
+      <c r="C44" s="6"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="F44" s="10"/>
-      <c r="G44" s="31" t="s">
+      <c r="F44" s="7"/>
+      <c r="G44" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H44" s="10"/>
-      <c r="I44" s="31" t="s">
+      <c r="H44" s="7"/>
+      <c r="I44" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="J44" s="10"/>
-      <c r="K44" s="32" t="s">
+      <c r="J44" s="7"/>
+      <c r="K44" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="45" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="9"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="9"/>
-      <c r="J45" s="10"/>
-      <c r="K45" s="11"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="22"/>
     </row>
     <row r="46" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="12"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9">
+      <c r="B46" s="34"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6">
         <v>60</v>
       </c>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9">
+      <c r="G46" s="6"/>
+      <c r="H46" s="6">
         <v>115</v>
       </c>
-      <c r="I46" s="9"/>
-      <c r="J46" s="9">
+      <c r="I46" s="6"/>
+      <c r="J46" s="6">
         <v>225</v>
       </c>
-      <c r="K46" s="11"/>
+      <c r="K46" s="22"/>
     </row>
     <row r="47" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="8"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="9"/>
-      <c r="J47" s="10"/>
-      <c r="K47" s="11"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="6"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="22"/>
     </row>
     <row r="48" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="8"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="10"/>
-      <c r="I48" s="9"/>
-      <c r="J48" s="10"/>
-      <c r="K48" s="11"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="22"/>
     </row>
-    <row r="49" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="13"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="33" t="s">
+    <row r="49" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="29"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="F49" s="15"/>
-      <c r="G49" s="33" t="s">
+      <c r="F49" s="31"/>
+      <c r="G49" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H49" s="15"/>
-      <c r="I49" s="33" t="s">
+      <c r="H49" s="31"/>
+      <c r="I49" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="J49" s="15"/>
-      <c r="K49" s="34" t="s">
+      <c r="J49" s="31"/>
+      <c r="K49" s="44" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix numbers of fixed slow-down tower in tower_upgrades.pdf
</commit_message>
<xml_diff>
--- a/assets/tower_upgrades.xlsx
+++ b/assets/tower_upgrades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daten\Projekte\pico\pico-bubble-towers\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377077C8-2F05-41CA-A015-93748907DB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4285E7DB-E35A-41CB-85FB-664C39E02DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{4E8ABA74-1C8E-408B-B6B2-4FB773843FD4}"/>
   </bookViews>
@@ -397,12 +397,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -445,9 +439,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -471,6 +462,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4874,67 +4874,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="16">
+      <c r="B1" s="42">
         <v>0</v>
       </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16">
+      <c r="C1" s="42"/>
+      <c r="D1" s="42">
         <v>1</v>
       </c>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16">
+      <c r="E1" s="42"/>
+      <c r="F1" s="42">
         <v>2</v>
       </c>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16">
+      <c r="G1" s="42"/>
+      <c r="H1" s="42">
         <v>3</v>
       </c>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16">
+      <c r="I1" s="42"/>
+      <c r="J1" s="42">
         <v>4</v>
       </c>
-      <c r="K1" s="16"/>
+      <c r="K1" s="42"/>
     </row>
     <row r="2" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:23" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="37">
+      <c r="B3" s="34">
         <v>10</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38">
+      <c r="C3" s="35"/>
+      <c r="D3" s="35">
         <v>18</v>
       </c>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38">
+      <c r="E3" s="35"/>
+      <c r="F3" s="35">
         <v>32</v>
       </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38">
+      <c r="G3" s="35"/>
+      <c r="H3" s="35">
         <v>90</v>
       </c>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38">
+      <c r="I3" s="35"/>
+      <c r="J3" s="35">
         <v>225</v>
       </c>
-      <c r="K3" s="39"/>
+      <c r="K3" s="36"/>
       <c r="M3" s="3"/>
       <c r="O3" s="3"/>
       <c r="Q3" s="3"/>
@@ -4946,7 +4946,7 @@
       <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="21"/>
+      <c r="B4" s="19"/>
       <c r="C4" s="6">
         <v>10</v>
       </c>
@@ -4963,7 +4963,7 @@
         <v>50</v>
       </c>
       <c r="J4" s="7"/>
-      <c r="K4" s="22">
+      <c r="K4" s="20">
         <v>70</v>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="21"/>
+      <c r="B5" s="19"/>
       <c r="C5" s="6">
         <v>16</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>26.6</v>
       </c>
       <c r="J5" s="7"/>
-      <c r="K5" s="22">
+      <c r="K5" s="20">
         <v>60</v>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="21"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="6">
         <v>10</v>
       </c>
@@ -5013,13 +5013,13 @@
         <v>10</v>
       </c>
       <c r="J6" s="7"/>
-      <c r="K6" s="22">
+      <c r="K6" s="20">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="34"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -5034,11 +5034,11 @@
       <c r="J7" s="6">
         <v>190</v>
       </c>
-      <c r="K7" s="22"/>
+      <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="19" t="s">
         <v>31</v>
       </c>
       <c r="C8" s="6"/>
@@ -5055,13 +5055,13 @@
         <v>35</v>
       </c>
       <c r="J8" s="6"/>
-      <c r="K8" s="22">
+      <c r="K8" s="20">
         <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>29</v>
       </c>
       <c r="C9" s="6"/>
@@ -5078,13 +5078,13 @@
         <v>21.3</v>
       </c>
       <c r="J9" s="6"/>
-      <c r="K9" s="22">
+      <c r="K9" s="20">
         <v>26.6</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="23"/>
+      <c r="B10" s="21"/>
       <c r="C10" s="8"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
@@ -5099,13 +5099,13 @@
         <v>5.3</v>
       </c>
       <c r="J10" s="8"/>
-      <c r="K10" s="24">
+      <c r="K10" s="22">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="37" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="5"/>
@@ -5122,11 +5122,11 @@
       <c r="J11" s="5">
         <v>150</v>
       </c>
-      <c r="K11" s="25"/>
+      <c r="K11" s="23"/>
     </row>
     <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="6"/>
@@ -5143,13 +5143,13 @@
         <v>75</v>
       </c>
       <c r="J12" s="7"/>
-      <c r="K12" s="22">
+      <c r="K12" s="20">
         <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="6"/>
@@ -5166,30 +5166,30 @@
         <v>24</v>
       </c>
       <c r="J13" s="7"/>
-      <c r="K13" s="22">
+      <c r="K13" s="20">
         <v>29.3</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="30">
+      <c r="F14" s="29"/>
+      <c r="G14" s="28">
         <v>13.3</v>
       </c>
-      <c r="H14" s="31"/>
-      <c r="I14" s="30">
+      <c r="H14" s="29"/>
+      <c r="I14" s="28">
         <v>13.3</v>
       </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="35">
+      <c r="J14" s="29"/>
+      <c r="K14" s="33">
         <v>13.3</v>
       </c>
     </row>
@@ -5197,27 +5197,27 @@
       <c r="A15" s="2"/>
     </row>
     <row r="16" spans="1:23" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19">
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17">
         <v>20</v>
       </c>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19">
+      <c r="E16" s="17"/>
+      <c r="F16" s="17">
         <v>40</v>
       </c>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19">
+      <c r="G16" s="17"/>
+      <c r="H16" s="17">
         <v>100</v>
       </c>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19">
+      <c r="I16" s="17"/>
+      <c r="J16" s="17">
         <v>250</v>
       </c>
-      <c r="K16" s="20"/>
+      <c r="K16" s="18"/>
     </row>
     <row r="17" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="21"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="7" t="s">
         <v>0</v>
       </c>
@@ -5234,12 +5234,12 @@
         <v>50</v>
       </c>
       <c r="J17" s="7"/>
-      <c r="K17" s="22">
+      <c r="K17" s="20">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="21"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="7" t="s">
         <v>1</v>
       </c>
@@ -5256,13 +5256,13 @@
         <v>33.299999999999997</v>
       </c>
       <c r="J18" s="7"/>
-      <c r="K18" s="22">
+      <c r="K18" s="20">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="21"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="7" t="s">
         <v>2</v>
       </c>
@@ -5279,13 +5279,13 @@
         <v>10</v>
       </c>
       <c r="J19" s="7"/>
-      <c r="K19" s="22">
+      <c r="K19" s="20">
         <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="34"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
@@ -5300,10 +5300,10 @@
       <c r="J20" s="6">
         <v>325</v>
       </c>
-      <c r="K20" s="22"/>
+      <c r="K20" s="20"/>
     </row>
     <row r="21" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="19" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="6"/>
@@ -5320,13 +5320,13 @@
         <v>60</v>
       </c>
       <c r="J21" s="7"/>
-      <c r="K21" s="22">
+      <c r="K21" s="20">
         <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="6"/>
@@ -5343,58 +5343,58 @@
         <v>24</v>
       </c>
       <c r="J22" s="7"/>
-      <c r="K22" s="22">
+      <c r="K22" s="20">
         <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31" t="s">
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F23" s="31"/>
-      <c r="G23" s="30">
+      <c r="F23" s="29"/>
+      <c r="G23" s="28">
         <v>13.3</v>
       </c>
-      <c r="H23" s="31"/>
-      <c r="I23" s="30">
+      <c r="H23" s="29"/>
+      <c r="I23" s="28">
         <v>13.3</v>
       </c>
-      <c r="J23" s="31"/>
-      <c r="K23" s="35">
+      <c r="J23" s="29"/>
+      <c r="K23" s="33">
         <v>13.3</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17">
         <v>35</v>
       </c>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19">
+      <c r="E25" s="17"/>
+      <c r="F25" s="17">
         <v>50</v>
       </c>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19">
+      <c r="G25" s="17"/>
+      <c r="H25" s="17">
         <v>115</v>
       </c>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19">
+      <c r="I25" s="17"/>
+      <c r="J25" s="17">
         <v>350</v>
       </c>
-      <c r="K25" s="20"/>
+      <c r="K25" s="18"/>
     </row>
     <row r="26" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="21"/>
+      <c r="B26" s="19"/>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="6">
@@ -5409,13 +5409,13 @@
         <v>50</v>
       </c>
       <c r="J26" s="7"/>
-      <c r="K26" s="22">
+      <c r="K26" s="20">
         <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="21"/>
+      <c r="B27" s="19"/>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
       <c r="E27" s="6">
@@ -5430,13 +5430,13 @@
         <v>18.600000000000001</v>
       </c>
       <c r="J27" s="7"/>
-      <c r="K27" s="22">
+      <c r="K27" s="20">
         <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="23"/>
+      <c r="B28" s="21"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8">
@@ -5451,12 +5451,12 @@
         <v>10</v>
       </c>
       <c r="J28" s="9"/>
-      <c r="K28" s="24">
+      <c r="K28" s="22">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="21" t="s">
+      <c r="B29" s="19" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="5"/>
@@ -5473,11 +5473,11 @@
       <c r="J29" s="5">
         <v>220</v>
       </c>
-      <c r="K29" s="25"/>
+      <c r="K29" s="23"/>
     </row>
     <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="19" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="6"/>
@@ -5494,12 +5494,12 @@
         <v>16</v>
       </c>
       <c r="J30" s="7"/>
-      <c r="K30" s="26" t="s">
+      <c r="K30" s="24" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C31" s="6"/>
@@ -5516,12 +5516,12 @@
         <v>16</v>
       </c>
       <c r="J31" s="7"/>
-      <c r="K31" s="26">
+      <c r="K31" s="24">
         <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="23"/>
+      <c r="B32" s="21"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -5530,10 +5530,10 @@
       <c r="H32" s="9"/>
       <c r="I32" s="8"/>
       <c r="J32" s="9"/>
-      <c r="K32" s="24"/>
+      <c r="K32" s="22"/>
     </row>
     <row r="33" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C33" s="5"/>
@@ -5550,10 +5550,10 @@
       <c r="J33" s="5">
         <v>180</v>
       </c>
-      <c r="K33" s="25"/>
+      <c r="K33" s="23"/>
     </row>
     <row r="34" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="19" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="6"/>
@@ -5564,10 +5564,10 @@
       <c r="H34" s="7"/>
       <c r="I34" s="6"/>
       <c r="J34" s="7"/>
-      <c r="K34" s="22"/>
+      <c r="K34" s="20"/>
     </row>
     <row r="35" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C35" s="6"/>
@@ -5577,60 +5577,60 @@
       </c>
       <c r="F35" s="7"/>
       <c r="G35" s="10">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="10">
-        <v>18.600000000000001</v>
+        <v>19</v>
       </c>
       <c r="J35" s="7"/>
-      <c r="K35" s="28">
+      <c r="K35" s="26">
         <v>24</v>
       </c>
     </row>
     <row r="36" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="29"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="32" t="s">
+      <c r="B36" s="27"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="F36" s="31"/>
-      <c r="G36" s="32" t="s">
+      <c r="F36" s="29"/>
+      <c r="G36" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="H36" s="31"/>
-      <c r="I36" s="32" t="s">
+      <c r="H36" s="29"/>
+      <c r="I36" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="J36" s="31"/>
-      <c r="K36" s="33" t="s">
+      <c r="J36" s="29"/>
+      <c r="K36" s="31" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="37" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="38" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="18"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19">
+      <c r="B38" s="16"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17">
         <v>40</v>
       </c>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19">
+      <c r="E38" s="17"/>
+      <c r="F38" s="17">
         <v>50</v>
       </c>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19">
+      <c r="G38" s="17"/>
+      <c r="H38" s="17">
         <v>90</v>
       </c>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19">
+      <c r="I38" s="17"/>
+      <c r="J38" s="17">
         <v>190</v>
       </c>
-      <c r="K38" s="20"/>
+      <c r="K38" s="18"/>
     </row>
     <row r="39" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="21"/>
+      <c r="B39" s="19"/>
       <c r="C39" s="14" t="s">
         <v>0</v>
       </c>
@@ -5647,12 +5647,12 @@
         <v>19</v>
       </c>
       <c r="J39" s="7"/>
-      <c r="K39" s="41" t="s">
+      <c r="K39" s="38" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="40" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="21"/>
+      <c r="B40" s="19"/>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
       <c r="E40" s="6"/>
@@ -5661,10 +5661,10 @@
       <c r="H40" s="7"/>
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
-      <c r="K40" s="22"/>
+      <c r="K40" s="20"/>
     </row>
     <row r="41" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="21"/>
+      <c r="B41" s="19"/>
       <c r="C41" s="6"/>
       <c r="D41" s="7"/>
       <c r="E41" s="6"/>
@@ -5673,10 +5673,10 @@
       <c r="H41" s="7"/>
       <c r="I41" s="6"/>
       <c r="J41" s="7"/>
-      <c r="K41" s="22"/>
+      <c r="K41" s="20"/>
     </row>
     <row r="42" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="34"/>
+      <c r="B42" s="32"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
@@ -5691,10 +5691,10 @@
       <c r="J42" s="6">
         <v>175</v>
       </c>
-      <c r="K42" s="22"/>
+      <c r="K42" s="20"/>
     </row>
     <row r="43" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="19" t="s">
         <v>23</v>
       </c>
       <c r="C43" s="6"/>
@@ -5705,10 +5705,10 @@
       <c r="H43" s="7"/>
       <c r="I43" s="6"/>
       <c r="J43" s="7"/>
-      <c r="K43" s="22"/>
+      <c r="K43" s="20"/>
     </row>
     <row r="44" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="21" t="s">
+      <c r="B44" s="19" t="s">
         <v>28</v>
       </c>
       <c r="C44" s="6"/>
@@ -5725,12 +5725,12 @@
         <v>21</v>
       </c>
       <c r="J44" s="7"/>
-      <c r="K44" s="42" t="s">
+      <c r="K44" s="39" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="45" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="21" t="s">
+      <c r="B45" s="19" t="s">
         <v>27</v>
       </c>
       <c r="C45" s="6"/>
@@ -5741,10 +5741,10 @@
       <c r="H45" s="7"/>
       <c r="I45" s="6"/>
       <c r="J45" s="7"/>
-      <c r="K45" s="22"/>
+      <c r="K45" s="20"/>
     </row>
     <row r="46" spans="2:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="34"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -5759,10 +5759,10 @@
       <c r="J46" s="6">
         <v>225</v>
       </c>
-      <c r="K46" s="22"/>
+      <c r="K46" s="20"/>
     </row>
     <row r="47" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="21"/>
+      <c r="B47" s="19"/>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
       <c r="E47" s="6"/>
@@ -5771,10 +5771,10 @@
       <c r="H47" s="7"/>
       <c r="I47" s="6"/>
       <c r="J47" s="7"/>
-      <c r="K47" s="22"/>
+      <c r="K47" s="20"/>
     </row>
     <row r="48" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="21"/>
+      <c r="B48" s="19"/>
       <c r="C48" s="6"/>
       <c r="D48" s="7"/>
       <c r="E48" s="6"/>
@@ -5783,25 +5783,25 @@
       <c r="H48" s="7"/>
       <c r="I48" s="6"/>
       <c r="J48" s="7"/>
-      <c r="K48" s="22"/>
+      <c r="K48" s="20"/>
     </row>
     <row r="49" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="29"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="31"/>
-      <c r="E49" s="43" t="s">
+      <c r="B49" s="27"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="F49" s="31"/>
-      <c r="G49" s="43" t="s">
+      <c r="F49" s="29"/>
+      <c r="G49" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="H49" s="31"/>
-      <c r="I49" s="43" t="s">
+      <c r="H49" s="29"/>
+      <c r="I49" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="J49" s="31"/>
-      <c r="K49" s="44" t="s">
+      <c r="J49" s="29"/>
+      <c r="K49" s="41" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>